<commit_message>
data(gold): freeze gold_labels.csv after A/B resolution
892 labels for 60 JDs. The 49 A/B disagreements were adjudicated with AI assistance (Claude) at annotator A's request; every decision and its reason is in resolution.xlsx. Rules R1-R5 from the resolution were added to ANNOTATION_GUIDE.md and applied to all 60 JDs. AGREEMENT.md keeps the pre-resolution figures (presence F1 0.867, kappa with negatives 0.763, importance weighted kappa 0.915).
</commit_message>
<xml_diff>
--- a/data/jd_dataset/gold/gold_workbook.xlsx
+++ b/data/jd_dataset/gold/gold_workbook.xlsx
@@ -4175,6 +4175,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
@@ -4366,7 +4367,7 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>NEW: Technical Support</t>
+          <t>NEW: IT Support</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
@@ -4384,7 +4385,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E40" s="8" t="n"/>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>renamed; guide rule R1 applied after the A/B resolution (AI-assisted, 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -6796,6 +6801,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
@@ -7238,18 +7244,58 @@
       <c r="E69" s="8" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="n"/>
-      <c r="B70" s="8" t="n"/>
-      <c r="C70" s="8" t="n"/>
-      <c r="D70" s="8" t="n"/>
-      <c r="E70" s="8" t="n"/>
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>Cloud Computing</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Windows, Linux, macOS, and cloud environments</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="n"/>
-      <c r="B71" s="8" t="n"/>
-      <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="n"/>
-      <c r="E71" s="8" t="n"/>
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Chain of Custody</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>chain-of-custody requirements</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n"/>
@@ -7689,6 +7735,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
@@ -8023,12 +8070,12 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>preferred</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Familiarity with security tools like SIEM, firewalls</t>
+          <t>Monitor security alerts and logs from various security tools such as SIEM (Security Information and Event Management) systems, firewalls</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -8036,12 +8083,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E45" s="8" t="n"/>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>importance preferred -&gt; required (duty); A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>NEW: Intrusion Detection</t>
+          <t>NEW: Intrusion Detection/Prevention</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
@@ -8059,21 +8110,65 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E46" s="8" t="n"/>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>renamed (R1); A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="n"/>
-      <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="n"/>
-      <c r="D47" s="8" t="n"/>
-      <c r="E47" s="8" t="n"/>
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Antivirus</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>antivirus</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="n"/>
-      <c r="B48" s="8" t="n"/>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
-      <c r="E48" s="8" t="n"/>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Operating Systems</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Basic understanding of network protocols, operating systems</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -10567,6 +10662,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
@@ -10952,7 +11048,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Learn and follow IT security practices?</t>
+          <t>Learn and follow IT security practices</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -10960,7 +11056,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E49" s="8" t="n"/>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>'?' resolved, preferred; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -10986,11 +11086,31 @@
       <c r="E50" s="8" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="n"/>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="8" t="n"/>
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access Management</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>preferred</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Learn and follow IT security practices, access control procedures</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
@@ -13052,6 +13172,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
@@ -13120,10 +13241,14 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>dropped: same sentence is Generative AI; guide rule R4 applied after the A/B resolution (AI-assisted, 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="47" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
@@ -20110,6 +20235,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
@@ -20598,18 +20724,58 @@
       <c r="E45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="n"/>
-      <c r="B46" s="8" t="n"/>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="8" t="n"/>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>NEW: UiPath</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>bonus</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>UiPath (RPA)</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="n"/>
-      <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="n"/>
-      <c r="D47" s="8" t="n"/>
-      <c r="E47" s="8" t="n"/>
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>NEW: IT Asset Management</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>IT asset management, inventory tracking</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -23843,6 +24009,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
@@ -24026,10 +24193,14 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>dropped: R&amp;D names an activity; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -24951,6 +25122,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
@@ -25106,7 +25278,7 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>* Artificial Intelligence</t>
+          <t>Participate in AI projects serving external customers</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
@@ -25114,7 +25286,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E84" s="8" t="n"/>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>evidence was a degree subject; replaced with a duty; guide rule R4 applied after the A/B resolution (AI-assisted, 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="17" customHeight="1">
       <c r="A85" s="8" t="inlineStr">
@@ -38433,6 +38609,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
@@ -38514,7 +38691,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>preferred</t>
+          <t>required</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -38527,7 +38704,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E39" s="8" t="n"/>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>importance preferred -&gt; required (duty); A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
@@ -38714,25 +38895,85 @@
       <c r="E47" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="n"/>
-      <c r="B48" s="8" t="n"/>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
-      <c r="E48" s="8" t="n"/>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>well-documented code</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="n"/>
-      <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="n"/>
-      <c r="D49" s="8" t="n"/>
-      <c r="E49" s="8" t="n"/>
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Backend Development</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Java-based backend services and APIs</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n"/>
-      <c r="B50" s="8" t="n"/>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Debugging</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Debug and troubleshoot application issues</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
@@ -42425,6 +42666,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
@@ -42631,10 +42873,14 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>dropped: under 'What you'll learn' (R2); A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -42683,11 +42929,31 @@
       <c r="E37" s="8" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="n"/>
-      <c r="B38" s="8" t="n"/>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="8" t="n"/>
-      <c r="E38" s="8" t="n"/>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Debugging</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Perform testing and debugging</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -51162,6 +51428,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
@@ -51443,11 +51710,31 @@
       <c r="E36" s="8" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n"/>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="8" t="n"/>
-      <c r="E37" s="8" t="n"/>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>NEW: Backend Development</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Expand and enhance existing backend services</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>added from B; A/B resolution, AI-assisted adjudication 2026-10-29, see resolution.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>

</xml_diff>